<commit_message>
Update field pengembalian pph, porongan berangkat siang, pulang awal
</commit_message>
<xml_diff>
--- a/src/assets/excel/template-payslip.xlsx
+++ b/src/assets/excel/template-payslip.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gbvh\src\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\PROJECT\gbvh\gbvh\src\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A05335-DE4E-4FC3-ACD4-6CB28A38E6F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5397F162-B7E6-4EE0-BBCF-C964C298B4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D20C10B8-C708-4404-8118-FB0D135168E9}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{D20C10B8-C708-4404-8118-FB0D135168E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>NIK</t>
   </si>
@@ -127,6 +127,15 @@
   </si>
   <si>
     <t>MONTH</t>
+  </si>
+  <si>
+    <t>POTONG_BERANGKAT_SIANG</t>
+  </si>
+  <si>
+    <t>POTONG_PULANG_AWAL</t>
+  </si>
+  <si>
+    <t>PENGEMBALIAN_PPH</t>
   </si>
 </sst>
 </file>
@@ -137,7 +146,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,8 +162,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -164,6 +180,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -195,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -216,6 +238,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,17 +557,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1C86984-557A-49A9-B90A-6FD29497B13B}">
-  <dimension ref="A1:AH1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AK1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="12" width="25.7109375" customWidth="1"/>
-    <col min="13" max="34" width="15.7109375" customWidth="1"/>
+    <col min="1" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="7" width="20.6640625" customWidth="1"/>
+    <col min="8" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="12" width="25.6640625" customWidth="1"/>
+    <col min="13" max="29" width="15.6640625" customWidth="1"/>
+    <col min="30" max="30" width="18.77734375" customWidth="1"/>
+    <col min="31" max="31" width="19" customWidth="1"/>
+    <col min="32" max="34" width="15.6640625" customWidth="1"/>
+    <col min="35" max="35" width="20" customWidth="1"/>
+    <col min="36" max="36" width="24.6640625" customWidth="1"/>
+    <col min="37" max="37" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -630,19 +661,28 @@
       <c r="AC1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AD1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AJ1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK1" s="5" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>